<commit_message>
Add dedicated Admin Panel for Layanan Inklusif (Braille & Disabilitas) and update Word/Excel guides with direct admin links
</commit_message>
<xml_diff>
--- a/AKIP_PKTJ_2025_LENGKAP_DENGAN_PATH_FILE.xlsx
+++ b/AKIP_PKTJ_2025_LENGKAP_DENGAN_PATH_FILE.xlsx
@@ -5770,7 +5770,7 @@
       </c>
       <c r="H93" s="52" t="inlineStr">
         <is>
-          <t>http://ppid.pktj.ac.id/admin/prosedur/sop-permintaan</t>
+          <t>http://ppid.pktj.ac.id/admin/layanan/aksesibilitas</t>
         </is>
       </c>
       <c r="I93" s="52" t="n"/>
@@ -5818,22 +5818,22 @@
       </c>
       <c r="E94" s="16" t="inlineStr">
         <is>
-          <t>Inovasi Formulir Layanan Braille, Audio Text-to-Speech, &amp; Video Panduan Bahasa Isyarat</t>
+          <t>Dokumen Formulir Permohonan &amp; Keberatan Huruf Braille serta Laporan Inovasi Layanan Ramah Disabilitas PPID PKTJ Tegal</t>
         </is>
       </c>
       <c r="F94" s="16" t="inlineStr">
         <is>
-          <t>Inovasi inklusivitas pelayanan informasi publik bagi penyandang disabilitas tunanetra, tunarungu, dan tunawicara.</t>
+          <t>Inovasi pemenuhan sarana aksesibilitas terpadu bagi penyandang disabilitas: Formulir Permohonan Braille, Pernyataan Keberatan Braille, Audio Text-to-Speech otomatis, serta Video Panduan Bahasa Isyarat (Bisindo).</t>
         </is>
       </c>
       <c r="G94" s="16" t="inlineStr">
         <is>
-          <t>FORMULIR PERMOHONAN BRAILLE.pdf &amp; Inovasi PPID.docx (Path: AKIP PKTJ 2025\Indikator I\FORMULIR PERMOHONAN INFORMASI PUBLIK BRAILE.pdf &amp; Inovasi PPID.docx)</t>
+          <t>FORMULIR PERMOHONAN BRAILE.pdf, PERNYATAAN KEBERATAN BRAILE.pdf, &amp; Inovasi PPID.docx (Path: AKIP PKTJ 2025\Indikator I\FORMULIR PERMOHONAN BRAILE.pdf, PERNYATAAN KEBERATAN BRAILE.pdf, &amp; Inovasi PPID.docx)</t>
         </is>
       </c>
       <c r="H94" s="52" t="inlineStr">
         <is>
-          <t>http://ppid.pktj.ac.id/admin/prosedur/sop-permintaan</t>
+          <t>http://ppid.pktj.ac.id/admin/layanan/aksesibilitas</t>
         </is>
       </c>
       <c r="I94" s="52" t="n"/>

</xml_diff>

<commit_message>
Update all Excel spreadsheet links to clickable hyperlinks with dedicated AKIP indicator URLs
</commit_message>
<xml_diff>
--- a/AKIP_PKTJ_2025_LENGKAP_DENGAN_PATH_FILE.xlsx
+++ b/AKIP_PKTJ_2025_LENGKAP_DENGAN_PATH_FILE.xlsx
@@ -17,7 +17,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d.m"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -150,6 +150,12 @@
       <color rgb="FFFF0000"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -191,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -342,6 +348,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -618,7 +627,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB1044"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.13" customWidth="1" style="53" min="1" max="1"/>
     <col width="8" customWidth="1" style="53" min="2" max="2"/>
@@ -861,7 +870,7 @@
           <t>A1.pdf (Path: AKIP PKTJ 2025\Indikator A\A1.pdf)</t>
         </is>
       </c>
-      <c r="H6" s="52" t="inlineStr">
+      <c r="H6" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/regulasi</t>
         </is>
@@ -917,7 +926,7 @@
           <t>A2.pdf (Path: AKIP PKTJ 2025\Indikator A\A2.pdf)</t>
         </is>
       </c>
-      <c r="H7" s="52" t="inlineStr">
+      <c r="H7" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/regulasi</t>
         </is>
@@ -973,7 +982,7 @@
           <t>A3.pdf (Path: AKIP PKTJ 2025\Indikator A\A3.pdf)</t>
         </is>
       </c>
-      <c r="H8" s="52" t="inlineStr">
+      <c r="H8" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/regulasi</t>
         </is>
@@ -1029,7 +1038,7 @@
           <t>Profil_PPID_PKTJ.pdf (Path: Tayang di Halaman Publik: /profil-ppid.html)</t>
         </is>
       </c>
-      <c r="H9" s="52" t="inlineStr">
+      <c r="H9" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/profil/edit/profil_singkat</t>
         </is>
@@ -1089,7 +1098,7 @@
           <t>Tugas_Fungsi_PPID.pdf (Path: Tayang di Halaman Publik: /profil-tugas-tanggung-jawab.html)</t>
         </is>
       </c>
-      <c r="H10" s="52" t="inlineStr">
+      <c r="H10" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/profil/edit/tugas_fungsi</t>
         </is>
@@ -1145,7 +1154,7 @@
           <t>A6.jpeg (Path: AKIP PKTJ 2025\Indikator A\A6.jpeg)</t>
         </is>
       </c>
-      <c r="H11" s="52" t="inlineStr">
+      <c r="H11" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/profil/edit/struktur_organisasi</t>
         </is>
@@ -1205,7 +1214,7 @@
           <t>Visi_Misi_PPID.pdf (Path: Tayang di Halaman Publik: /profil-visi-misi.html)</t>
         </is>
       </c>
-      <c r="H12" s="52" t="inlineStr">
+      <c r="H12" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/profil/edit/visi_misi</t>
         </is>
@@ -1261,9 +1270,9 @@
           <t>A8.JPG (Path: AKIP PKTJ 2025\Indikator A\A8.JPG)</t>
         </is>
       </c>
-      <c r="H13" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/berkala/create</t>
+      <c r="H13" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/A8/edit</t>
         </is>
       </c>
       <c r="I13" s="52" t="n"/>
@@ -1317,9 +1326,9 @@
           <t>A9 2024.jpg &amp; A9 2025.jpg (Path: AKIP PKTJ 2025\Indikator A\A9\A9 2024.jpg &amp; A9 2025.jpg)</t>
         </is>
       </c>
-      <c r="H14" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/berkala/create</t>
+      <c r="H14" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/A9/edit</t>
         </is>
       </c>
       <c r="I14" s="52" t="n"/>
@@ -1423,9 +1432,9 @@
           <t>B1-B4.pdf (Halaman POK Anggaran) (Path: AKIP PKTJ 2025\Indikator B\B1-B4.pdf)</t>
         </is>
       </c>
-      <c r="H16" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/berkala/create</t>
+      <c r="H16" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/B1/edit</t>
         </is>
       </c>
       <c r="I16" s="52" t="n"/>
@@ -1483,7 +1492,7 @@
           <t>B1-B4.pdf (Halaman Laporan Kegiatan) (Path: AKIP PKTJ 2025\Indikator B\B1-B4.pdf)</t>
         </is>
       </c>
-      <c r="H17" s="52" t="inlineStr">
+      <c r="H17" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/layanan/laporan-layanan</t>
         </is>
@@ -1543,9 +1552,9 @@
           <t>B1-B4.pdf (Halaman Alur Koordinasi) (Path: AKIP PKTJ 2025\Indikator B\B1-B4.pdf)</t>
         </is>
       </c>
-      <c r="H18" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/prosedur/sop-keberatan</t>
+      <c r="H18" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/prosedur/sop-sengketa</t>
         </is>
       </c>
       <c r="I18" s="52" t="n"/>
@@ -1603,9 +1612,9 @@
           <t>B1-B4.pdf (Halaman Usulan DIP/DIK) (Path: AKIP PKTJ 2025\Indikator B\B1-B4.pdf)</t>
         </is>
       </c>
-      <c r="H19" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/setiap-saat/create</t>
+      <c r="H19" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/B4/edit</t>
         </is>
       </c>
       <c r="I19" s="52" t="n"/>
@@ -1663,9 +1672,9 @@
           <t>B5.pdf / B5.jpeg / B5.png (Path: AKIP PKTJ 2025\Indikator B\B5\B5.pdf)</t>
         </is>
       </c>
-      <c r="H20" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/berkala/create</t>
+      <c r="H20" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/B5/edit</t>
         </is>
       </c>
       <c r="I20" s="52" t="inlineStr">
@@ -1779,7 +1788,7 @@
           <t>C1.png / C2.JPG / DSC06430-6435.JPG (Path: AKIP PKTJ 2025\Indikator C\C1.png &amp; C2.JPG)</t>
         </is>
       </c>
-      <c r="H22" s="52" t="inlineStr">
+      <c r="H22" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/layanan/maklumat-pelayanan</t>
         </is>
@@ -1835,7 +1844,7 @@
           <t>C3.pdf (Path: AKIP PKTJ 2025\Indikator C\C3.pdf)</t>
         </is>
       </c>
-      <c r="H23" s="52" t="inlineStr">
+      <c r="H23" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/prosedur/sop-permintaan</t>
         </is>
@@ -1891,7 +1900,7 @@
           <t>Register_Permohonan_NIHIL.pdf (Path: AKIP PKTJ 2025\Indikator C\Register_Permohonan_NIHIL.pdf)</t>
         </is>
       </c>
-      <c r="H24" s="52" t="inlineStr">
+      <c r="H24" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/layanan/laporan-layanan</t>
         </is>
@@ -1951,7 +1960,7 @@
           <t>C5.pdf / C5.JPG / C5.png (Path: AKIP PKTJ 2025\Indikator C\C5\C5.pdf)</t>
         </is>
       </c>
-      <c r="H25" s="52" t="inlineStr">
+      <c r="H25" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/layanan/maklumat-pelayanan</t>
         </is>
@@ -2007,7 +2016,7 @@
           <t>C6.pdf / C6.JPG / C6.png (Path: AKIP PKTJ 2025\Indikator C\C6\C6.pdf)</t>
         </is>
       </c>
-      <c r="H26" s="52" t="inlineStr">
+      <c r="H26" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/layanan/maklumat-pelayanan</t>
         </is>
@@ -2067,7 +2076,7 @@
           <t>Banner_SOP_Layanan.jpg (Path: AKIP PKTJ 2025\Indikator C\Banner_SOP_Layanan.jpg)</t>
         </is>
       </c>
-      <c r="H27" s="52" t="inlineStr">
+      <c r="H27" s="54" t="inlineStr">
         <is>
           <t>http://ppid.pktj.ac.id/admin/prosedur/sop-permintaan</t>
         </is>
@@ -2128,9 +2137,9 @@
 </t>
         </is>
       </c>
-      <c r="H28" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/menu</t>
+      <c r="H28" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/prosedur/sop-keberatan</t>
         </is>
       </c>
       <c r="I28" s="52" t="n"/>
@@ -2188,9 +2197,9 @@
           <t>D1.pdf (Path: AKIP PKTJ 2025\Indikator D\D1.pdf)</t>
         </is>
       </c>
-      <c r="H29" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/menu</t>
+      <c r="H29" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/prosedur/sop-sengketa</t>
         </is>
       </c>
       <c r="I29" s="52" t="n"/>
@@ -2244,9 +2253,9 @@
           <t>D2.pdf / D3.pdf / D4.pdf (Path: AKIP PKTJ 2025\Indikator D\D2.pdf &amp; D3.pdf)</t>
         </is>
       </c>
-      <c r="H30" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/berkala</t>
+      <c r="H30" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/prosedur/sop-penetapan</t>
         </is>
       </c>
       <c r="I30" s="52" t="n"/>
@@ -2354,9 +2363,9 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="H32" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/laporan-layanan</t>
+      <c r="H32" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/layanan/aksesibilitas</t>
         </is>
       </c>
       <c r="I32" s="52" t="n"/>
@@ -2415,9 +2424,9 @@
           <t>E.1.3.png / E2.pdf / E3.pdf / E4.pdf (Path: AKIP PKTJ 2025\Indikator E\E2.pdf &amp; E3.pdf)</t>
         </is>
       </c>
-      <c r="H33" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/laporan-layanan</t>
+      <c r="H33" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/layanan/aksesibilitas</t>
         </is>
       </c>
       <c r="I33" s="52" t="n"/>
@@ -2471,9 +2480,9 @@
           <t>E6.pdf / E6a.jpg / E6b.jpg / E7.pdf (Path: AKIP PKTJ 2025\Indikator E\E6.pdf &amp; E7.pdf)</t>
         </is>
       </c>
-      <c r="H34" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/laporan-layanan</t>
+      <c r="H34" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/layanan/aksesibilitas</t>
         </is>
       </c>
       <c r="I34" s="52" t="n"/>
@@ -2523,9 +2532,9 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="H35" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/berkala</t>
+      <c r="H35" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/layanan/aksesibilitas</t>
         </is>
       </c>
       <c r="I35" s="52" t="n"/>
@@ -2579,9 +2588,9 @@
           <t>F1.pdf (Path: AKIP PKTJ 2025\Indikator F\F1.pdf)</t>
         </is>
       </c>
-      <c r="H36" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/berkala/create</t>
+      <c r="H36" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/layanan/aksesibilitas</t>
         </is>
       </c>
       <c r="I36" s="52" t="n"/>
@@ -2693,9 +2702,9 @@
           <t>F3.xlsx / Laptah_PKTJ.pdf (Path: AKIP PKTJ 2025\Indikator F\F3.xlsx)</t>
         </is>
       </c>
-      <c r="H38" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/berkala/create</t>
+      <c r="H38" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/dashboard</t>
         </is>
       </c>
       <c r="I38" s="52" t="n"/>
@@ -2917,9 +2926,9 @@
           <t>F7.pdf (Path: AKIP PKTJ 2025\Indikator F\F7.pdf)</t>
         </is>
       </c>
-      <c r="H42" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/berkala/create</t>
+      <c r="H42" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/dashboard</t>
         </is>
       </c>
       <c r="I42" s="52" t="n"/>
@@ -2973,9 +2982,9 @@
           <t>F8.xlsx / Chart_Kepegawaian.png (Path: AKIP PKTJ 2025\Indikator F\F8.xlsx)</t>
         </is>
       </c>
-      <c r="H43" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/berkala</t>
+      <c r="H43" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/permohonan-informasi</t>
         </is>
       </c>
       <c r="I43" s="52" t="n"/>
@@ -3029,9 +3038,9 @@
           <t>F9.xlsx (Path: AKIP PKTJ 2025\Indikator F\F9.xlsx)</t>
         </is>
       </c>
-      <c r="H44" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/berkala/create</t>
+      <c r="H44" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/keberatan</t>
         </is>
       </c>
       <c r="I44" s="52" t="n"/>
@@ -3081,7 +3090,11 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="H45" s="52" t="n"/>
+      <c r="H45" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/kontak</t>
+        </is>
+      </c>
       <c r="I45" s="52" t="n"/>
       <c r="J45" s="52" t="n"/>
       <c r="K45" s="52" t="n"/>
@@ -3133,7 +3146,11 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="H46" s="52" t="n"/>
+      <c r="H46" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/kontak</t>
+        </is>
+      </c>
       <c r="I46" s="52" t="n"/>
       <c r="J46" s="52" t="n"/>
       <c r="K46" s="52" t="n"/>
@@ -3186,7 +3203,11 @@
 https://pktj.ac.id/tentang/94-informasi-berkala</t>
         </is>
       </c>
-      <c r="H47" s="52" t="n"/>
+      <c r="H47" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/layanan/laporan-layanan</t>
+        </is>
+      </c>
       <c r="I47" s="52" t="n"/>
       <c r="J47" s="52" t="n"/>
       <c r="K47" s="52" t="n"/>
@@ -3296,9 +3317,9 @@
           <t>F12.pdf (Halaman KAK) (Path: AKIP PKTJ 2025\Indikator F\F12.pdf)</t>
         </is>
       </c>
-      <c r="H49" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/daftar-informasi/create</t>
+      <c r="H49" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/F1/edit</t>
         </is>
       </c>
       <c r="I49" s="52" t="n"/>
@@ -3352,9 +3373,9 @@
           <t>F12.pdf (Halaman HPS) (Path: AKIP PKTJ 2025\Indikator F\F12.pdf)</t>
         </is>
       </c>
-      <c r="H50" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/daftar-informasi/create</t>
+      <c r="H50" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/F2/edit</t>
         </is>
       </c>
       <c r="I50" s="52" t="n"/>
@@ -3408,9 +3429,9 @@
           <t>F12.pdf (Halaman Spektek) (Path: AKIP PKTJ 2025\Indikator F\F12.pdf)</t>
         </is>
       </c>
-      <c r="H51" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/daftar-informasi/create</t>
+      <c r="H51" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/pejabat</t>
         </is>
       </c>
       <c r="I51" s="52" t="n"/>
@@ -3464,9 +3485,9 @@
           <t>F12.pdf (Halaman Rancangan Kontrak) (Path: AKIP PKTJ 2025\Indikator F\F12.pdf)</t>
         </is>
       </c>
-      <c r="H52" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/daftar-informasi/create</t>
+      <c r="H52" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/F4/edit</t>
         </is>
       </c>
       <c r="I52" s="52" t="n"/>
@@ -3520,9 +3541,9 @@
           <t>F12.pdf (Halaman LDK) (Path: AKIP PKTJ 2025\Indikator F\F12.pdf)</t>
         </is>
       </c>
-      <c r="H53" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/daftar-informasi/create</t>
+      <c r="H53" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/F5/edit</t>
         </is>
       </c>
       <c r="I53" s="52" t="n"/>
@@ -3580,9 +3601,9 @@
           <t>F12.pdf (Halaman LDP) (Path: AKIP PKTJ 2025\Indikator F\F12.pdf)</t>
         </is>
       </c>
-      <c r="H54" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/daftar-informasi/create</t>
+      <c r="H54" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/F6/edit</t>
         </is>
       </c>
       <c r="I54" s="52" t="n"/>
@@ -3636,9 +3657,9 @@
           <t>F12.pdf (Halaman BoQ) (Path: AKIP PKTJ 2025\Indikator F\F12.pdf)</t>
         </is>
       </c>
-      <c r="H55" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/daftar-informasi/create</t>
+      <c r="H55" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/F7/edit</t>
         </is>
       </c>
       <c r="I55" s="52" t="n"/>
@@ -3692,9 +3713,9 @@
           <t>F12.pdf (Halaman Jadwal/Lokasi) (Path: AKIP PKTJ 2025\Indikator F\F12.pdf)</t>
         </is>
       </c>
-      <c r="H56" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/daftar-informasi/create</t>
+      <c r="H56" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/F8/edit</t>
         </is>
       </c>
       <c r="I56" s="52" t="n"/>
@@ -3748,9 +3769,9 @@
           <t>F12.pdf (Halaman Gambar Rancang) (Path: AKIP PKTJ 2025\Indikator F\F12.pdf)</t>
         </is>
       </c>
-      <c r="H57" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/daftar-informasi/create</t>
+      <c r="H57" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/F9/edit</t>
         </is>
       </c>
       <c r="I57" s="52" t="n"/>
@@ -3804,9 +3825,9 @@
           <t>F12.pdf (Halaman Lingkungan) (Path: AKIP PKTJ 2025\Indikator F\F12.pdf)</t>
         </is>
       </c>
-      <c r="H58" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/daftar-informasi/create</t>
+      <c r="H58" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/F10/edit</t>
         </is>
       </c>
       <c r="I58" s="52" t="n"/>
@@ -5486,9 +5507,9 @@
           <t>G2.pdf (Path: AKIP PKTJ 2025\Indikator G\G2.pdf)</t>
         </is>
       </c>
-      <c r="H88" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/setiap-saat/create</t>
+      <c r="H88" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/G1/edit</t>
         </is>
       </c>
       <c r="I88" s="52" t="n"/>
@@ -5542,9 +5563,9 @@
           <t>Surat Masuk &amp; Keluar 2023-2025.pdf (Path: AKIP PKTJ 2025\Indikator G\G3\Surat Masuk tahun 2023-2025.pdf &amp; Surat Keluar.pdf)</t>
         </is>
       </c>
-      <c r="H89" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/setiap-saat/create</t>
+      <c r="H89" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/G2/edit</t>
         </is>
       </c>
       <c r="I89" s="52" t="n"/>
@@ -5598,9 +5619,9 @@
           <t>Laporan_BMN_PKTJ_2025_Audited.pdf (Path: AKIP PKTJ 2025\Indikator G\Laporan_BMN_PKTJ_2025.pdf)</t>
         </is>
       </c>
-      <c r="H90" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/informasi/setiap-saat/create</t>
+      <c r="H90" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/G3/edit</t>
         </is>
       </c>
       <c r="I90" s="52" t="n"/>
@@ -5768,9 +5789,9 @@
           <t>https://pktj.ac.id/tentang/96-informasi-serta-merta</t>
         </is>
       </c>
-      <c r="H93" s="52" t="inlineStr">
-        <is>
-          <t>http://ppid.pktj.ac.id/admin/layanan/aksesibilitas</t>
+      <c r="H93" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/akip/H1/edit</t>
         </is>
       </c>
       <c r="I93" s="52" t="n"/>
@@ -5883,8 +5904,10 @@
         </is>
       </c>
       <c r="G95" s="16" t="n"/>
-      <c r="H95" s="52" t="n">
-        <v>43</v>
+      <c r="H95" s="54" t="inlineStr">
+        <is>
+          <t>http://ppid.pktj.ac.id/admin/layanan/aksesibilitas</t>
+        </is>
       </c>
       <c r="I95" s="52" t="inlineStr">
         <is>
@@ -34398,100 +34421,150 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId146"/>
   </hyperlinks>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>